<commit_message>
[Foldering] UIStartScene 연결 완료
</commit_message>
<xml_diff>
--- a/Assets/Resources/Excels/ItemSheets.xlsx
+++ b/Assets/Resources/Excels/ItemSheets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Project\In_You\Assets\Resources\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{394AADD1-A84F-4773-BA23-B7852BC907C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{487F5774-4222-473D-A7F1-FA164187F8ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F2D3F8C6-91EA-41DC-95B7-AEFA1AA84CB8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{F2D3F8C6-91EA-41DC-95B7-AEFA1AA84CB8}"/>
   </bookViews>
   <sheets>
     <sheet name="ItemSheets" sheetId="1" r:id="rId1"/>
@@ -81,25 +81,27 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>add</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>물</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>물약</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Consumable</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>calcType</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>duration</t>
-  </si>
-  <si>
-    <t>calcType</t>
-  </si>
-  <si>
-    <t>add</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>물</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>물약</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Consumable</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -498,13 +500,13 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" t="s">
         <v>14</v>
-      </c>
-      <c r="C2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" t="s">
-        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -537,13 +539,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{083C45C4-908C-498D-A565-9594F5573554}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="17.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -554,13 +556,13 @@
         <v>10</v>
       </c>
       <c r="D1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E1" t="s">
-        <v>12</v>
+        <v>16</v>
+      </c>
+      <c r="F1" t="s">
+        <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>11</v>
       </c>
@@ -568,10 +570,10 @@
         <v>11</v>
       </c>
       <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2" t="s">
-        <v>13</v>
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>